<commit_message>
feat: mid-month update June 2026 (through 2026-06-16)
Jun 2026 partial data added to raw_2026:
- Outage: EU SAST Aviator Jun 8 19:11-19:13 GMT (2 min)
- Outage: AMS SAST Aviator Jun 9 21:09-21:11 GMT (2 min)
- Service Degradation: AMS Portal+API Jun 9 16:55 - Jun 10 22:44 GMT (tracked, excluded from uptime)
All times converted from BST (GMT+1). De-duped incidents: 20 -> 22. YTD unchanged (Jan-May complete).

https://claude.ai/code/session_012cvNt9u1ZM5WgpyCJq7uXC
</commit_message>
<xml_diff>
--- a/FoD_Uptime_Report_2026.xlsx
+++ b/FoD_Uptime_Report_2026.xlsx
@@ -545,14 +545,14 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>1. Jan: 4 outages (5 min); Feb: 3 outages (9 min); Mar: 7 outages (57 min); Apr: 4 outages (25 min); May: 2 outages (4 min)</t>
+          <t>1. Jan: 4 outages (5 min); Feb: 3 outages (9 min); Mar: 7 outages (57 min); Apr: 4 outages (25 min); May: 2 outages (4 min); Jun (partial thru Jun 16): 2 outages (4 min)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Completed Months: January - May 2026 (June in progress)</t>
+          <t>Completed Months: January - May 2026 (June partial through Jun 16, 2026)</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>3. SAST Aviator (EU/AMS) continued brief outage pattern: Mar 11, 13, 17, 18; Apr 9 EU SAST 2 min; May 9 EU SAST 2 min, May 10 AMS SAST 2 min</t>
+          <t>3. SAST Aviator (EU/AMS) continued brief outage pattern: Mar 11, 13, 17, 18; Apr 9 EU SAST 2 min; May 9 EU SAST 2 min, May 10 AMS SAST 2 min; Jun 8 EU SAST 2 min, Jun 9 AMS SAST 2 min</t>
         </is>
       </c>
     </row>
@@ -734,21 +734,21 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>2*</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>4*</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>0.0*</t>
+          <t>0.07*</t>
         </is>
       </c>
       <c r="E20" s="8" t="n">
-        <v>1</v>
+        <v>0.9999074074074074</v>
       </c>
     </row>
     <row r="21">
@@ -935,7 +935,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>* June 2026 is in progress. Will be finalized after June 30, 2026.</t>
+          <t>* June 2026 is in progress (partial through June 16, 2026). Will be finalized after June 30, 2026.</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Last updated: June 2, 2026 (May 2026 finalized; no outage events May 17-31; maintenance added: APAC/SGP May 27 BST, EMEA May 27-28 BST, EU/FedRAMP/AMS May 28 BST; service degradation May 14-26 AMS added).</t>
+          <t>Last updated: June 16, 2026 (mid-month update; Jun 2026 partial data added through Jun 16: 2 outages (EU SAST Aviator Jun 8 2 min, AMS SAST Aviator Jun 9 2 min) + AMS service degradation Jun 9-10; times converted from BST to GMT).</t>
         </is>
       </c>
     </row>
@@ -2138,7 +2138,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Last updated: June 2, 2026</t>
+          <t>Last updated: June 16, 2026</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
         <v>0.9999551971326165</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>1</v>
+        <v>0.9999537037037037</v>
       </c>
       <c r="H20" s="14" t="inlineStr">
         <is>
@@ -3141,7 +3141,7 @@
         <v>0.9999551971326165</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>1</v>
+        <v>0.9999537037037037</v>
       </c>
       <c r="H21" s="14" t="inlineStr">
         <is>
@@ -5124,7 +5124,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Month in progress. Will be finalized after June 30, 2026.</t>
+          <t>Month in progress. Partial data through June 16, 2026. Will be finalized after June 30, 2026.</t>
         </is>
       </c>
     </row>
@@ -5167,7 +5167,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>100.0000%</t>
+          <t>99.9907%</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5264,120 +5264,120 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T03:57:00Z</t>
+          <t>2026-06-09T21:09:00Z</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 5:43 AM GMT</t>
+          <t>Jun 09, 2026 9:11 PM GMT</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T03:57:00Z</t>
+          <t>2026-06-09T16:55:00Z</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 5:43 AM GMT</t>
+          <t>Jun 10, 2026 10:44 PM GMT</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>106</v>
+        <v>1789</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T02:06:00Z</t>
+          <t>2026-06-09T16:55:00Z</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 3:03 AM GMT</t>
+          <t>Jun 10, 2026 10:44 PM GMT</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>57</v>
+        <v>1789</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T02:06:00Z</t>
+          <t>2026-06-08T19:11:00Z</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 3:03 AM GMT</t>
+          <t>Jun 08, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>57</v>
+        <v>2</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
@@ -5389,21 +5389,21 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T01:07:00Z</t>
+          <t>2026-05-28T03:57:00Z</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:40 AM GMT</t>
+          <t>May 28, 2026 5:43 AM GMT</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -5419,21 +5419,21 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T01:07:00Z</t>
+          <t>2026-05-28T03:57:00Z</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:40 AM GMT</t>
+          <t>May 28, 2026 5:43 AM GMT</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -5449,21 +5449,21 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T23:50:00Z</t>
+          <t>2026-05-28T02:06:00Z</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:06 AM GMT</t>
+          <t>May 28, 2026 3:03 AM GMT</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -5479,21 +5479,21 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T23:50:00Z</t>
+          <t>2026-05-28T02:06:00Z</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:06 AM GMT</t>
+          <t>May 28, 2026 3:03 AM GMT</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -5509,21 +5509,21 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-28T01:07:00Z</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:40 AM GMT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -5539,21 +5539,21 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-28T01:07:00Z</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:40 AM GMT</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
@@ -5569,21 +5569,21 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-27T23:50:00Z</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:06 AM GMT</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -5599,21 +5599,21 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-27T23:50:00Z</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:06 AM GMT</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -5624,26 +5624,26 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-05-14T12:22:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>May 26, 2026 1:56 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>17374</v>
+        <v>122</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -5654,26 +5654,26 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-05-14T12:22:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>May 26, 2026 1:56 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>17374</v>
+        <v>122</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -5684,26 +5684,26 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2026-05-13T14:30:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>May 13, 2026 2:35 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>5</v>
+        <v>122</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -5714,26 +5714,26 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-05-13T14:30:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>May 13, 2026 2:35 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>5</v>
+        <v>122</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -5744,26 +5744,26 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>2026-05-11T14:06:00Z</t>
+          <t>2026-05-14T12:22:00Z</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>May 12, 2026 1:19 AM GMT</t>
+          <t>May 26, 2026 1:56 PM GMT</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>673</v>
+        <v>17374</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -5774,26 +5774,26 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-05-11T14:06:00Z</t>
+          <t>2026-05-14T12:22:00Z</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>May 12, 2026 1:19 AM GMT</t>
+          <t>May 26, 2026 1:56 PM GMT</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>673</v>
+        <v>17374</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -5804,26 +5804,26 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2026-05-10T21:09:00Z</t>
+          <t>2026-05-13T14:30:00Z</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>May 10, 2026 9:11 PM GMT</t>
+          <t>May 13, 2026 2:35 PM GMT</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -5834,26 +5834,26 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-05-09T19:11:00Z</t>
+          <t>2026-05-13T14:30:00Z</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>May 09, 2026 7:13 PM GMT</t>
+          <t>May 13, 2026 2:35 PM GMT</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -5869,21 +5869,21 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08T09:39:00Z</t>
+          <t>2026-05-11T14:06:00Z</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 11:51 AM GMT</t>
+          <t>May 12, 2026 1:19 AM GMT</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>132</v>
+        <v>673</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -5899,21 +5899,21 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08T09:39:00Z</t>
+          <t>2026-05-11T14:06:00Z</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 11:51 AM GMT</t>
+          <t>May 12, 2026 1:19 AM GMT</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>132</v>
+        <v>673</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -5924,26 +5924,26 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2026-05-07T19:05:00Z</t>
+          <t>2026-05-10T21:09:00Z</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 6:20 PM GMT</t>
+          <t>May 10, 2026 9:11 PM GMT</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1395</v>
+        <v>2</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -5954,26 +5954,26 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-05-07T19:05:00Z</t>
+          <t>2026-05-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 6:20 PM GMT</t>
+          <t>May 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1395</v>
+        <v>2</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -5989,21 +5989,21 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04T17:22:00Z</t>
+          <t>2026-05-08T09:39:00Z</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 6:34 PM GMT</t>
+          <t>May 08, 2026 11:51 AM GMT</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -6019,21 +6019,21 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04T17:22:00Z</t>
+          <t>2026-05-08T09:39:00Z</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 6:34 PM GMT</t>
+          <t>May 08, 2026 11:51 AM GMT</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -6044,17 +6044,17 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T03:17:00Z</t>
+          <t>2026-05-07T19:05:00Z</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 5:59 AM GMT</t>
+          <t>May 08, 2026 6:20 PM GMT</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -6063,28 +6063,28 @@
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>162</v>
+        <v>1395</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T03:17:00Z</t>
+          <t>2026-05-07T19:05:00Z</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 5:59 AM GMT</t>
+          <t>May 08, 2026 6:20 PM GMT</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -6093,11 +6093,11 @@
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>162</v>
+        <v>1395</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -6109,25 +6109,25 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:52:00Z</t>
+          <t>2026-05-04T17:22:00Z</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 2:10 AM GMT</t>
+          <t>May 04, 2026 6:34 PM GMT</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -6139,25 +6139,25 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:52:00Z</t>
+          <t>2026-05-04T17:22:00Z</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 2:10 AM GMT</t>
+          <t>May 04, 2026 6:34 PM GMT</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -6169,21 +6169,21 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:20:00Z</t>
+          <t>2026-04-30T03:17:00Z</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:48 AM GMT</t>
+          <t>Apr 30, 2026 5:59 AM GMT</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>88</v>
+        <v>162</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -6199,21 +6199,21 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:20:00Z</t>
+          <t>2026-04-30T03:17:00Z</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:48 AM GMT</t>
+          <t>Apr 30, 2026 5:59 AM GMT</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>88</v>
+        <v>162</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -6229,21 +6229,21 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T22:53:00Z</t>
+          <t>2026-04-30T00:52:00Z</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 12:06 AM GMT</t>
+          <t>Apr 30, 2026 2:10 AM GMT</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -6259,21 +6259,21 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T22:53:00Z</t>
+          <t>2026-04-30T00:52:00Z</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 12:06 AM GMT</t>
+          <t>Apr 30, 2026 2:10 AM GMT</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -6289,21 +6289,21 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-30T00:20:00Z</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 1:48 AM GMT</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>273</v>
+        <v>88</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
@@ -6319,21 +6319,21 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-30T00:20:00Z</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 1:48 AM GMT</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>273</v>
+        <v>88</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
@@ -6349,21 +6349,21 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-29T22:53:00Z</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 12:06 AM GMT</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>273</v>
+        <v>73</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
@@ -6379,21 +6379,21 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-29T22:53:00Z</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 12:06 AM GMT</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>273</v>
+        <v>73</v>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
@@ -6409,21 +6409,21 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24T18:12:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Apr 24, 2026 10:14 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>242</v>
+        <v>273</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
@@ -6439,21 +6439,21 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24T18:12:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Apr 24, 2026 10:14 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>242</v>
+        <v>273</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
@@ -6464,26 +6464,26 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>2026-04-22T16:29:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 4:21 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>17272</v>
+        <v>273</v>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
@@ -6494,26 +6494,26 @@
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-04-22T16:29:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 4:21 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>17272</v>
+        <v>273</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
@@ -6529,21 +6529,21 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>2026-04-21T20:43:00Z</t>
+          <t>2026-04-24T18:12:00Z</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Apr 22, 2026 4:30 PM GMT</t>
+          <t>Apr 24, 2026 10:14 PM GMT</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1187</v>
+        <v>242</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
@@ -6559,21 +6559,21 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-04-21T20:43:00Z</t>
+          <t>2026-04-24T18:12:00Z</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Apr 22, 2026 4:30 PM GMT</t>
+          <t>Apr 24, 2026 10:14 PM GMT</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>1187</v>
+        <v>242</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
@@ -6584,17 +6584,17 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17T22:57:00Z</t>
+          <t>2026-04-22T16:29:00Z</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Apr 20, 2026 10:21 PM GMT</t>
+          <t>May 04, 2026 4:21 PM GMT</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
@@ -6603,7 +6603,7 @@
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>4284</v>
+        <v>17272</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
@@ -6614,17 +6614,17 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17T22:57:00Z</t>
+          <t>2026-04-22T16:29:00Z</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Apr 20, 2026 10:21 PM GMT</t>
+          <t>May 04, 2026 4:21 PM GMT</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
@@ -6633,7 +6633,7 @@
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>4284</v>
+        <v>17272</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
@@ -6644,17 +6644,17 @@
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2026-04-16T14:28:00Z</t>
+          <t>2026-04-21T20:43:00Z</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 2:38 PM GMT</t>
+          <t>Apr 22, 2026 4:30 PM GMT</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -6663,7 +6663,7 @@
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>10</v>
+        <v>1187</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
@@ -6674,17 +6674,17 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-04-16T14:26:00Z</t>
+          <t>2026-04-21T20:43:00Z</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 2:36 PM GMT</t>
+          <t>Apr 22, 2026 4:30 PM GMT</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
@@ -6693,7 +6693,7 @@
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>10</v>
+        <v>1187</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
@@ -6709,21 +6709,21 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>2026-04-10T20:56:00Z</t>
+          <t>2026-04-17T22:57:00Z</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Apr 10, 2026 10:32 PM GMT</t>
+          <t>Apr 20, 2026 10:21 PM GMT</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>96</v>
+        <v>4284</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
@@ -6739,21 +6739,21 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T21:04:00Z</t>
+          <t>2026-04-17T22:57:00Z</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 9:34 PM GMT</t>
+          <t>Apr 20, 2026 10:21 PM GMT</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>30</v>
+        <v>4284</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
@@ -6769,21 +6769,21 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T19:11:00Z</t>
+          <t>2026-04-16T14:28:00Z</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 7:13 PM GMT</t>
+          <t>Apr 16, 2026 2:38 PM GMT</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
@@ -6794,26 +6794,26 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T18:04:00Z</t>
+          <t>2026-04-16T14:26:00Z</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 9:35 PM GMT</t>
+          <t>Apr 16, 2026 2:36 PM GMT</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>211</v>
+        <v>10</v>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
@@ -6824,26 +6824,26 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2026-04-08T04:10:00Z</t>
+          <t>2026-04-10T20:56:00Z</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Apr 08, 2026 4:12 AM GMT</t>
+          <t>Apr 10, 2026 10:32 PM GMT</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
@@ -6854,26 +6854,26 @@
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-04-08T04:09:00Z</t>
+          <t>2026-04-09T21:04:00Z</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Apr 08, 2026 4:12 AM GMT</t>
+          <t>Apr 09, 2026 9:34 PM GMT</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
@@ -6884,26 +6884,26 @@
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>2026-04-07T18:03:00Z</t>
+          <t>2026-04-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Apr 07, 2026 7:21 PM GMT</t>
+          <t>Apr 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
@@ -6919,21 +6919,21 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-09T18:04:00Z</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 09, 2026 9:35 PM GMT</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>50</v>
+        <v>211</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
@@ -6944,17 +6944,17 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-08T04:10:00Z</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -6963,7 +6963,7 @@
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
@@ -6974,60 +6974,60 @@
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-08T04:09:00Z</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>203</v>
+        <v>3</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-07T18:03:00Z</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 07, 2026 7:21 PM GMT</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>203</v>
+        <v>78</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -7039,25 +7039,25 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -7069,25 +7069,25 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -7099,21 +7099,21 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>123</v>
+        <v>203</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
@@ -7129,21 +7129,21 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>123</v>
+        <v>203</v>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
@@ -7159,21 +7159,21 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E65" s="5" t="n">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
@@ -7189,21 +7189,21 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
@@ -7219,21 +7219,21 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T21:04:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 10:34 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
@@ -7249,21 +7249,21 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T17:44:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 6:26 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
@@ -7279,21 +7279,21 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
@@ -7309,21 +7309,21 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E70" s="5" t="n">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
@@ -7334,17 +7334,17 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T00:43:00Z</t>
+          <t>2026-03-20T21:04:00Z</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 12:46 AM GMT</t>
+          <t>Mar 20, 2026 10:34 PM GMT</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
@@ -7353,7 +7353,7 @@
         </is>
       </c>
       <c r="E71" s="5" t="n">
-        <v>3</v>
+        <v>90</v>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
@@ -7369,21 +7369,21 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-20T17:44:00Z</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 20, 2026 6:26 PM GMT</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>198</v>
+        <v>42</v>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
@@ -7399,21 +7399,21 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
@@ -7424,26 +7424,26 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T19:46:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Mar 17, 2026 7:48 PM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
@@ -7459,12 +7459,12 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>2026-03-13T00:37:00Z</t>
+          <t>2026-03-18T00:43:00Z</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Mar 13, 2026 12:41 AM GMT</t>
+          <t>Mar 18, 2026 12:46 AM GMT</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
@@ -7473,7 +7473,7 @@
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
@@ -7484,26 +7484,26 @@
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>2026-03-11T23:50:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Mar 11, 2026 11:54 PM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>4</v>
+        <v>198</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
@@ -7519,21 +7519,21 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>164</v>
+        <v>198</v>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
@@ -7544,26 +7544,26 @@
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-17T19:46:00Z</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 17, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>164</v>
+        <v>2</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
@@ -7574,26 +7574,26 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-13T00:37:00Z</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 13, 2026 12:41 AM GMT</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E79" s="5" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
@@ -7604,26 +7604,26 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-11T23:50:00Z</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 11, 2026 11:54 PM GMT</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E80" s="5" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
@@ -7639,21 +7639,21 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E81" s="5" t="n">
-        <v>87</v>
+        <v>164</v>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
@@ -7669,21 +7669,21 @@
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>87</v>
+        <v>164</v>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
@@ -7699,21 +7699,21 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
@@ -7729,21 +7729,21 @@
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E84" s="5" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
@@ -7759,21 +7759,21 @@
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E85" s="5" t="n">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
@@ -7789,21 +7789,21 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E86" s="5" t="n">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
@@ -7814,26 +7814,26 @@
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 5:02 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E87" s="5" t="n">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
@@ -7844,26 +7844,26 @@
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 4:56 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E88" s="5" t="n">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
@@ -7874,26 +7874,26 @@
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:44:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 3:15 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E89" s="5" t="n">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
@@ -7904,26 +7904,26 @@
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:42:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:44 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E90" s="5" t="n">
-        <v>2</v>
+        <v>95</v>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
@@ -7939,12 +7939,12 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:41:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:42 PM GMT</t>
+          <t>Mar 02, 2026 5:02 PM GMT</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
@@ -7953,7 +7953,7 @@
         </is>
       </c>
       <c r="E91" s="5" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
@@ -7969,17 +7969,17 @@
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>2026-02-26T16:39:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Feb 26, 2026 4:44 PM GMT</t>
+          <t>Mar 02, 2026 4:56 PM GMT</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E92" s="5" t="n">
@@ -7987,123 +7987,123 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-02T14:44:00Z</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 02, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>207</v>
+        <v>31</v>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-02T14:42:00Z</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 02, 2026 2:44 PM GMT</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E94" s="5" t="n">
-        <v>207</v>
+        <v>2</v>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-03-02T14:41:00Z</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Mar 02, 2026 2:42 PM GMT</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E95" s="5" t="n">
-        <v>159</v>
+        <v>1</v>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-02-26T16:39:00Z</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Feb 26, 2026 4:44 PM GMT</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E96" s="5" t="n">
-        <v>159</v>
+        <v>5</v>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
@@ -8114,26 +8114,26 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>2026-02-15T19:46:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Feb 15, 2026 7:48 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E97" s="5" t="n">
-        <v>2</v>
+        <v>207</v>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
@@ -8144,26 +8144,26 @@
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14T22:07:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Feb 14, 2026 10:09 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E98" s="5" t="n">
-        <v>2</v>
+        <v>207</v>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
@@ -8179,21 +8179,21 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E99" s="5" t="n">
-        <v>282</v>
+        <v>159</v>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
@@ -8209,21 +8209,21 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E100" s="5" t="n">
-        <v>282</v>
+        <v>159</v>
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
@@ -8234,26 +8234,26 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-02-15T19:46:00Z</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Feb 15, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E101" s="5" t="n">
-        <v>127</v>
+        <v>2</v>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
@@ -8264,26 +8264,26 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-02-14T22:07:00Z</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Feb 14, 2026 10:09 PM GMT</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E102" s="5" t="n">
-        <v>127</v>
+        <v>2</v>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
@@ -8299,21 +8299,21 @@
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E103" s="5" t="n">
-        <v>98</v>
+        <v>282</v>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
@@ -8329,21 +8329,21 @@
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E104" s="5" t="n">
-        <v>98</v>
+        <v>282</v>
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
@@ -8359,21 +8359,21 @@
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E105" s="5" t="n">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
@@ -8389,21 +8389,21 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E106" s="5" t="n">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
@@ -8419,25 +8419,25 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E107" s="5" t="n">
-        <v>4234</v>
+        <v>98</v>
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -8449,85 +8449,85 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E108" s="5" t="n">
-        <v>4234</v>
+        <v>98</v>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:46:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:47 PM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E109" s="5" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:45:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:46 PM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E110" s="5" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -8539,21 +8539,21 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E111" s="5" t="n">
-        <v>1595</v>
+        <v>4234</v>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
@@ -8569,21 +8569,21 @@
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C112" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E112" s="5" t="n">
-        <v>1595</v>
+        <v>4234</v>
       </c>
       <c r="F112" s="5" t="inlineStr">
         <is>
@@ -8594,26 +8594,26 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T16:24:00Z</t>
+          <t>2026-01-27T14:46:00Z</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Jan 20, 2026 3:26 AM GMT</t>
+          <t>Jan 27, 2026 2:47 PM GMT</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E113" s="5" t="n">
-        <v>4982</v>
+        <v>1</v>
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
@@ -8629,17 +8629,17 @@
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T15:14:00Z</t>
+          <t>2026-01-27T14:45:00Z</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:15 PM GMT</t>
+          <t>Jan 27, 2026 2:46 PM GMT</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E114" s="5" t="n">
@@ -8659,21 +8659,21 @@
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T21:13:00Z</t>
+          <t>2026-01-23T23:57:00Z</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:03 PM GMT</t>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E115" s="5" t="n">
-        <v>1070</v>
+        <v>1595</v>
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
@@ -8684,26 +8684,26 @@
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T04:24:00Z</t>
+          <t>2026-01-23T23:57:00Z</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>Jan 15, 2026 4:25 AM GMT</t>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand - Vulncat</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E116" s="5" t="n">
-        <v>1</v>
+        <v>1595</v>
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
@@ -8714,17 +8714,17 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>2026-01-10T15:08:00Z</t>
+          <t>2026-01-16T16:24:00Z</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Jan 10, 2026 3:10 PM GMT</t>
+          <t>Jan 20, 2026 3:26 AM GMT</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr">
@@ -8733,7 +8733,7 @@
         </is>
       </c>
       <c r="E117" s="5" t="n">
-        <v>2</v>
+        <v>4982</v>
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
@@ -8744,26 +8744,26 @@
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-01-16T15:14:00Z</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Jan 16, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E118" s="5" t="n">
-        <v>140</v>
+        <v>1</v>
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
@@ -8779,21 +8779,21 @@
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-01-15T21:13:00Z</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Jan 16, 2026 3:03 PM GMT</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E119" s="5" t="n">
-        <v>140</v>
+        <v>1070</v>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
@@ -8804,26 +8804,26 @@
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-15T04:24:00Z</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Jan 15, 2026 4:25 AM GMT</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand - Vulncat</t>
         </is>
       </c>
       <c r="E120" s="5" t="n">
-        <v>137</v>
+        <v>1</v>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
@@ -8834,26 +8834,26 @@
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-10T15:08:00Z</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Jan 10, 2026 3:10 PM GMT</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E121" s="5" t="n">
-        <v>137</v>
+        <v>2</v>
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
@@ -8869,21 +8869,21 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T00:24:00Z</t>
+          <t>2026-01-08T04:54:00Z</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 1:02 AM GMT</t>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E122" s="5" t="n">
-        <v>38</v>
+        <v>140</v>
       </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
@@ -8899,32 +8899,152 @@
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
+          <t>2026-01-08T04:54:00Z</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - AMS</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="n">
+        <v>140</v>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D124" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E124" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E125" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B126" s="5" t="inlineStr">
+        <is>
           <t>2026-01-08T00:24:00Z</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
+      <c r="C126" s="5" t="inlineStr">
         <is>
           <t>Jan 08, 2026 1:02 AM GMT</t>
         </is>
       </c>
-      <c r="D123" s="5" t="inlineStr">
+      <c r="D126" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
+        </is>
+      </c>
+      <c r="E126" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T00:24:00Z</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 1:02 AM GMT</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
         <is>
           <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
-      <c r="E123" s="5" t="n">
+      <c r="E127" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="F123" s="5" t="inlineStr">
+      <c r="F127" s="5" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="11" t="inlineStr">
-        <is>
-          <t>Report revised: June 02, 2026</t>
+    <row r="128">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>Report revised: June 16, 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: mid-month update July 2026 (through 2026-07-16)
3 outages added for Jul 1-15: Jul 6 APAC Portal 6 min, Jul 7 APAC API 7 min,
Jul 8 AMS SAST Aviator 4 min. All times converted from BST to GMT.
months_complete unchanged (Jun still last finalized month). No fabricated data.
</commit_message>
<xml_diff>
--- a/FoD_Uptime_Report_2026.xlsx
+++ b/FoD_Uptime_Report_2026.xlsx
@@ -754,21 +754,21 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>3*</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>0*</t>
+          <t>17*</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>0.0*</t>
+          <t>0.28*</t>
         </is>
       </c>
       <c r="E21" s="8" t="n">
-        <v>1</v>
+        <v>0.9996191756272401</v>
       </c>
     </row>
     <row r="22">
@@ -928,7 +928,7 @@
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>* July 2026 is in progress. Will be finalized after July 31, 2026.</t>
+          <t>* July 2026 is in progress (partial through July 16, 2026). Will be finalized after July 31, 2026.</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1052,90 +1052,90 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>2026-06-27T00:18:00Z</t>
+          <t>2026-07-08T16:34:00Z</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Jun 27, 2026 12:40 AM GMT</t>
+          <t>Jul 08, 2026 4:38 PM GMT</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>2026-06-27T00:18:00Z</t>
+          <t>2026-07-07T22:42:00Z</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Jun 27, 2026 12:40 AM GMT</t>
+          <t>Jul 07, 2026 10:49 PM GMT</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T18:24:00Z</t>
+          <t>2026-07-06T16:05:00Z</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 9:36 PM GMT</t>
+          <t>Jul 06, 2026 4:11 PM GMT</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
-        <v>192</v>
+        <v>6</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
@@ -1147,21 +1147,21 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T18:24:00Z</t>
+          <t>2026-06-27T00:18:00Z</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 9:36 PM GMT</t>
+          <t>Jun 27, 2026 12:40 AM GMT</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>192</v>
+        <v>22</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1177,21 +1177,21 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T18:23:00Z</t>
+          <t>2026-06-27T00:18:00Z</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 9:07 PM GMT</t>
+          <t>Jun 27, 2026 12:40 AM GMT</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>164</v>
+        <v>22</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -1207,21 +1207,21 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T18:23:00Z</t>
+          <t>2026-06-25T18:24:00Z</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 9:07 PM GMT</t>
+          <t>Jun 25, 2026 9:36 PM GMT</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
-        <v>164</v>
+        <v>192</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -1237,21 +1237,21 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T04:06:00Z</t>
+          <t>2026-06-25T18:24:00Z</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 8:18 AM GMT</t>
+          <t>Jun 25, 2026 9:36 PM GMT</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
-        <v>252</v>
+        <v>192</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -1267,21 +1267,21 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T04:06:00Z</t>
+          <t>2026-06-25T18:23:00Z</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 8:18 AM GMT</t>
+          <t>Jun 25, 2026 9:07 PM GMT</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
-        <v>252</v>
+        <v>164</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -1297,21 +1297,21 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T00:26:00Z</t>
+          <t>2026-06-25T18:23:00Z</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 1:08 AM GMT</t>
+          <t>Jun 25, 2026 9:07 PM GMT</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>42</v>
+        <v>164</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -1327,21 +1327,21 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-25T00:26:00Z</t>
+          <t>2026-06-25T04:06:00Z</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 1:08 AM GMT</t>
+          <t>Jun 25, 2026 8:18 AM GMT</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
-        <v>42</v>
+        <v>252</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
@@ -1357,21 +1357,21 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T23:19:00Z</t>
+          <t>2026-06-25T04:06:00Z</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 12:57 AM GMT</t>
+          <t>Jun 25, 2026 8:18 AM GMT</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>98</v>
+        <v>252</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
@@ -1387,21 +1387,21 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T23:19:00Z</t>
+          <t>2026-06-25T00:26:00Z</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 12:57 AM GMT</t>
+          <t>Jun 25, 2026 1:08 AM GMT</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>98</v>
+        <v>42</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -1417,21 +1417,21 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T13:57:00Z</t>
+          <t>2026-06-25T00:26:00Z</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Jun 24, 2026 3:20 PM GMT</t>
+          <t>Jun 25, 2026 1:08 AM GMT</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>83</v>
+        <v>42</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -1447,21 +1447,21 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T13:57:00Z</t>
+          <t>2026-06-24T23:19:00Z</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Jun 24, 2026 3:20 PM GMT</t>
+          <t>Jun 25, 2026 12:57 AM GMT</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -1477,21 +1477,21 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T13:51:00Z</t>
+          <t>2026-06-24T23:19:00Z</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Jun 24, 2026 3:47 PM GMT</t>
+          <t>Jun 25, 2026 12:57 AM GMT</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1507,21 +1507,21 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24T13:51:00Z</t>
+          <t>2026-06-24T13:57:00Z</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Jun 24, 2026 3:47 PM GMT</t>
+          <t>Jun 24, 2026 3:20 PM GMT</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>116</v>
+        <v>83</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -1537,21 +1537,21 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-23T17:55:00Z</t>
+          <t>2026-06-24T13:57:00Z</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Jun 23, 2026 6:45 PM GMT</t>
+          <t>Jun 24, 2026 3:20 PM GMT</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -1567,21 +1567,21 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2026-06-22T21:08:00Z</t>
+          <t>2026-06-24T13:51:00Z</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Jun 22, 2026 9:40 PM GMT</t>
+          <t>Jun 24, 2026 3:47 PM GMT</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E19" s="5" t="n">
-        <v>32</v>
+        <v>116</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -1592,26 +1592,26 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-11T11:50:00Z</t>
+          <t>2026-06-24T13:51:00Z</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 1:23 PM GMT</t>
+          <t>Jun 24, 2026 3:47 PM GMT</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E20" s="5" t="n">
-        <v>20253</v>
+        <v>116</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -1622,26 +1622,26 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-06-11T11:50:00Z</t>
+          <t>2026-06-23T17:55:00Z</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Jun 25, 2026 1:23 PM GMT</t>
+          <t>Jun 23, 2026 6:45 PM GMT</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>20253</v>
+        <v>50</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -1652,17 +1652,17 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-09T21:09:00Z</t>
+          <t>2026-06-22T21:08:00Z</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Jun 09, 2026 9:11 PM GMT</t>
+          <t>Jun 22, 2026 9:40 PM GMT</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>2026-06-09T16:55:00Z</t>
+          <t>2026-06-11T11:50:00Z</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Jun 10, 2026 10:44 PM GMT</t>
+          <t>Jun 25, 2026 1:23 PM GMT</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>1789</v>
+        <v>20253</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -1717,12 +1717,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-09T16:55:00Z</t>
+          <t>2026-06-11T11:50:00Z</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Jun 10, 2026 10:44 PM GMT</t>
+          <t>Jun 25, 2026 1:23 PM GMT</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1789</v>
+        <v>20253</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1747,17 +1747,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-08T19:11:00Z</t>
+          <t>2026-06-09T21:09:00Z</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Jun 08, 2026 7:13 PM GMT</t>
+          <t>Jun 09, 2026 9:11 PM GMT</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
@@ -1772,17 +1772,17 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>2026-06-04T21:22:00Z</t>
+          <t>2026-06-09T16:55:00Z</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Jun 05, 2026 12:25 PM GMT</t>
+          <t>Jun 10, 2026 10:44 PM GMT</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="E26" s="5" t="n">
-        <v>903</v>
+        <v>1789</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -1802,17 +1802,17 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2026-06-04T21:22:00Z</t>
+          <t>2026-06-09T16:55:00Z</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Jun 05, 2026 12:25 PM GMT</t>
+          <t>Jun 10, 2026 10:44 PM GMT</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1821,7 +1821,7 @@
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>903</v>
+        <v>1789</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -1832,30 +1832,30 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T03:57:00Z</t>
+          <t>2026-06-08T19:11:00Z</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 5:43 AM GMT</t>
+          <t>Jun 08, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
@@ -1867,25 +1867,25 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T03:57:00Z</t>
+          <t>2026-06-04T21:22:00Z</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 5:43 AM GMT</t>
+          <t>Jun 05, 2026 12:25 PM GMT</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
-        <v>106</v>
+        <v>903</v>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
@@ -1897,25 +1897,25 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T02:06:00Z</t>
+          <t>2026-06-04T21:22:00Z</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 3:03 AM GMT</t>
+          <t>Jun 05, 2026 12:25 PM GMT</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v>57</v>
+        <v>903</v>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>2026-05</t>
+          <t>2026-06</t>
         </is>
       </c>
     </row>
@@ -1927,21 +1927,21 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T02:06:00Z</t>
+          <t>2026-05-28T03:57:00Z</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 3:03 AM GMT</t>
+          <t>May 28, 2026 5:43 AM GMT</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
-        <v>57</v>
+        <v>106</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
@@ -1957,21 +1957,21 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T01:07:00Z</t>
+          <t>2026-05-28T03:57:00Z</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:40 AM GMT</t>
+          <t>May 28, 2026 5:43 AM GMT</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -1987,21 +1987,21 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>2026-05-28T01:07:00Z</t>
+          <t>2026-05-28T02:06:00Z</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:40 AM GMT</t>
+          <t>May 28, 2026 3:03 AM GMT</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
@@ -2017,21 +2017,21 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T23:50:00Z</t>
+          <t>2026-05-28T02:06:00Z</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:06 AM GMT</t>
+          <t>May 28, 2026 3:03 AM GMT</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
-        <v>76</v>
+        <v>57</v>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
@@ -2047,21 +2047,21 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T23:50:00Z</t>
+          <t>2026-05-28T01:07:00Z</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>May 28, 2026 1:06 AM GMT</t>
+          <t>May 28, 2026 1:40 AM GMT</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>76</v>
+        <v>33</v>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
@@ -2077,21 +2077,21 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-28T01:07:00Z</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:40 AM GMT</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E36" s="5" t="n">
-        <v>122</v>
+        <v>33</v>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
@@ -2107,21 +2107,21 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-27T23:50:00Z</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:06 AM GMT</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
@@ -2137,21 +2137,21 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>2026-05-27T15:12:00Z</t>
+          <t>2026-05-27T23:50:00Z</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>May 27, 2026 5:14 PM GMT</t>
+          <t>May 28, 2026 1:06 AM GMT</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>122</v>
+        <v>76</v>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
@@ -2192,26 +2192,26 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>2026-05-14T12:22:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>May 26, 2026 1:56 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E40" s="5" t="n">
-        <v>17374</v>
+        <v>122</v>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
@@ -2222,26 +2222,26 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>2026-05-14T12:22:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>May 26, 2026 1:56 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E41" s="5" t="n">
-        <v>17374</v>
+        <v>122</v>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
@@ -2252,26 +2252,26 @@
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>2026-05-13T14:30:00Z</t>
+          <t>2026-05-27T15:12:00Z</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>May 13, 2026 2:35 PM GMT</t>
+          <t>May 27, 2026 5:14 PM GMT</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
-        <v>5</v>
+        <v>122</v>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
@@ -2287,21 +2287,21 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>2026-05-13T14:30:00Z</t>
+          <t>2026-05-14T12:22:00Z</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>May 13, 2026 2:35 PM GMT</t>
+          <t>May 26, 2026 1:56 PM GMT</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E43" s="5" t="n">
-        <v>5</v>
+        <v>17374</v>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
@@ -2312,26 +2312,26 @@
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>2026-05-11T14:06:00Z</t>
+          <t>2026-05-14T12:22:00Z</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>May 12, 2026 1:19 AM GMT</t>
+          <t>May 26, 2026 1:56 PM GMT</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
-        <v>673</v>
+        <v>17374</v>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
@@ -2342,26 +2342,26 @@
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>2026-05-11T14:06:00Z</t>
+          <t>2026-05-13T14:30:00Z</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>May 12, 2026 1:19 AM GMT</t>
+          <t>May 13, 2026 2:35 PM GMT</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>673</v>
+        <v>5</v>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
@@ -2372,26 +2372,26 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>2026-05-10T21:09:00Z</t>
+          <t>2026-05-13T14:30:00Z</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>May 10, 2026 9:11 PM GMT</t>
+          <t>May 13, 2026 2:35 PM GMT</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E46" s="5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
@@ -2402,26 +2402,26 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>2026-05-09T19:11:00Z</t>
+          <t>2026-05-11T14:06:00Z</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>May 09, 2026 7:13 PM GMT</t>
+          <t>May 12, 2026 1:19 AM GMT</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>2</v>
+        <v>673</v>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
@@ -2437,21 +2437,21 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08T09:39:00Z</t>
+          <t>2026-05-11T14:06:00Z</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 11:51 AM GMT</t>
+          <t>May 12, 2026 1:19 AM GMT</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>132</v>
+        <v>673</v>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
@@ -2462,26 +2462,26 @@
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>2026-05-08T09:39:00Z</t>
+          <t>2026-05-10T21:09:00Z</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 11:51 AM GMT</t>
+          <t>May 10, 2026 9:11 PM GMT</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E49" s="5" t="n">
-        <v>132</v>
+        <v>2</v>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
@@ -2492,26 +2492,26 @@
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>2026-05-07T19:05:00Z</t>
+          <t>2026-05-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 6:20 PM GMT</t>
+          <t>May 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E50" s="5" t="n">
-        <v>1395</v>
+        <v>2</v>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
@@ -2522,26 +2522,26 @@
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>2026-05-07T19:05:00Z</t>
+          <t>2026-05-08T09:39:00Z</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>May 08, 2026 6:20 PM GMT</t>
+          <t>May 08, 2026 11:51 AM GMT</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>1395</v>
+        <v>132</v>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
@@ -2557,21 +2557,21 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04T17:22:00Z</t>
+          <t>2026-05-08T09:39:00Z</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 6:34 PM GMT</t>
+          <t>May 08, 2026 11:51 AM GMT</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
@@ -2582,26 +2582,26 @@
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>2026-05-04T17:22:00Z</t>
+          <t>2026-05-07T19:05:00Z</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 6:34 PM GMT</t>
+          <t>May 08, 2026 6:20 PM GMT</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>72</v>
+        <v>1395</v>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
@@ -2612,30 +2612,30 @@
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T03:17:00Z</t>
+          <t>2026-05-07T19:05:00Z</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 5:59 AM GMT</t>
+          <t>May 08, 2026 6:20 PM GMT</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>162</v>
+        <v>1395</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -2647,25 +2647,25 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T03:17:00Z</t>
+          <t>2026-05-04T17:22:00Z</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 5:59 AM GMT</t>
+          <t>May 04, 2026 6:34 PM GMT</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>162</v>
+        <v>72</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -2677,25 +2677,25 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:52:00Z</t>
+          <t>2026-05-04T17:22:00Z</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 2:10 AM GMT</t>
+          <t>May 04, 2026 6:34 PM GMT</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>2026-04</t>
+          <t>2026-05</t>
         </is>
       </c>
     </row>
@@ -2707,21 +2707,21 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:52:00Z</t>
+          <t>2026-04-30T03:17:00Z</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 2:10 AM GMT</t>
+          <t>Apr 30, 2026 5:59 AM GMT</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>78</v>
+        <v>162</v>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
@@ -2737,21 +2737,21 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:20:00Z</t>
+          <t>2026-04-30T03:17:00Z</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:48 AM GMT</t>
+          <t>Apr 30, 2026 5:59 AM GMT</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E58" s="5" t="n">
-        <v>88</v>
+        <v>162</v>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
@@ -2767,21 +2767,21 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>2026-04-30T00:20:00Z</t>
+          <t>2026-04-30T00:52:00Z</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 1:48 AM GMT</t>
+          <t>Apr 30, 2026 2:10 AM GMT</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
@@ -2797,21 +2797,21 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T22:53:00Z</t>
+          <t>2026-04-30T00:52:00Z</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 12:06 AM GMT</t>
+          <t>Apr 30, 2026 2:10 AM GMT</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
@@ -2827,21 +2827,21 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T22:53:00Z</t>
+          <t>2026-04-30T00:20:00Z</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Apr 30, 2026 12:06 AM GMT</t>
+          <t>Apr 30, 2026 1:48 AM GMT</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
@@ -2857,21 +2857,21 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-30T00:20:00Z</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 1:48 AM GMT</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>273</v>
+        <v>88</v>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
@@ -2887,21 +2887,21 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-29T22:53:00Z</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 12:06 AM GMT</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>273</v>
+        <v>73</v>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
@@ -2917,21 +2917,21 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>2026-04-29T15:45:00Z</t>
+          <t>2026-04-29T22:53:00Z</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Apr 29, 2026 8:18 PM GMT</t>
+          <t>Apr 30, 2026 12:06 AM GMT</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>273</v>
+        <v>73</v>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E65" s="5" t="n">
@@ -2977,21 +2977,21 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24T18:12:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Apr 24, 2026 10:14 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>242</v>
+        <v>273</v>
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
@@ -3007,21 +3007,21 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>2026-04-24T18:12:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Apr 24, 2026 10:14 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>242</v>
+        <v>273</v>
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
@@ -3032,26 +3032,26 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>2026-04-22T16:29:00Z</t>
+          <t>2026-04-29T15:45:00Z</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 4:21 PM GMT</t>
+          <t>Apr 29, 2026 8:18 PM GMT</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>17272</v>
+        <v>273</v>
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
@@ -3062,26 +3062,26 @@
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>2026-04-22T16:29:00Z</t>
+          <t>2026-04-24T18:12:00Z</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>May 04, 2026 4:21 PM GMT</t>
+          <t>Apr 24, 2026 10:14 PM GMT</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>17272</v>
+        <v>242</v>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
@@ -3097,21 +3097,21 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>2026-04-21T20:43:00Z</t>
+          <t>2026-04-24T18:12:00Z</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Apr 22, 2026 4:30 PM GMT</t>
+          <t>Apr 24, 2026 10:14 PM GMT</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E70" s="5" t="n">
-        <v>1187</v>
+        <v>242</v>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
@@ -3122,26 +3122,26 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>2026-04-21T20:43:00Z</t>
+          <t>2026-04-22T16:29:00Z</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Apr 22, 2026 4:30 PM GMT</t>
+          <t>May 04, 2026 4:21 PM GMT</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E71" s="5" t="n">
-        <v>1187</v>
+        <v>17272</v>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
@@ -3152,26 +3152,26 @@
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17T22:57:00Z</t>
+          <t>2026-04-22T16:29:00Z</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Apr 20, 2026 10:21 PM GMT</t>
+          <t>May 04, 2026 4:21 PM GMT</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>4284</v>
+        <v>17272</v>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
@@ -3187,21 +3187,21 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>2026-04-17T22:57:00Z</t>
+          <t>2026-04-21T20:43:00Z</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Apr 20, 2026 10:21 PM GMT</t>
+          <t>Apr 22, 2026 4:30 PM GMT</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>4284</v>
+        <v>1187</v>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
@@ -3212,26 +3212,26 @@
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>2026-04-16T14:28:00Z</t>
+          <t>2026-04-21T20:43:00Z</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 2:38 PM GMT</t>
+          <t>Apr 22, 2026 4:30 PM GMT</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EU</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E74" s="5" t="n">
-        <v>10</v>
+        <v>1187</v>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
@@ -3242,26 +3242,26 @@
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>2026-04-16T14:26:00Z</t>
+          <t>2026-04-17T22:57:00Z</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>Apr 16, 2026 2:36 PM GMT</t>
+          <t>Apr 20, 2026 10:21 PM GMT</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EU</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>10</v>
+        <v>4284</v>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
@@ -3277,21 +3277,21 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>2026-04-10T20:56:00Z</t>
+          <t>2026-04-17T22:57:00Z</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Apr 10, 2026 10:32 PM GMT</t>
+          <t>Apr 20, 2026 10:21 PM GMT</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>96</v>
+        <v>4284</v>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
@@ -3302,26 +3302,26 @@
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T21:04:00Z</t>
+          <t>2026-04-16T14:28:00Z</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 9:34 PM GMT</t>
+          <t>Apr 16, 2026 2:38 PM GMT</t>
         </is>
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - EU</t>
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
@@ -3337,21 +3337,21 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T19:11:00Z</t>
+          <t>2026-04-16T14:26:00Z</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 7:13 PM GMT</t>
+          <t>Apr 16, 2026 2:36 PM GMT</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - EU</t>
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F78" s="5" t="inlineStr">
         <is>
@@ -3367,21 +3367,21 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>2026-04-09T18:04:00Z</t>
+          <t>2026-04-10T20:56:00Z</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Apr 09, 2026 9:35 PM GMT</t>
+          <t>Apr 10, 2026 10:32 PM GMT</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E79" s="5" t="n">
-        <v>211</v>
+        <v>96</v>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
@@ -3392,26 +3392,26 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>2026-04-08T04:10:00Z</t>
+          <t>2026-04-09T21:04:00Z</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Apr 08, 2026 4:12 AM GMT</t>
+          <t>Apr 09, 2026 9:34 PM GMT</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E80" s="5" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
@@ -3427,21 +3427,21 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>2026-04-08T04:09:00Z</t>
+          <t>2026-04-09T19:11:00Z</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Apr 08, 2026 4:12 AM GMT</t>
+          <t>Apr 09, 2026 7:13 PM GMT</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E81" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
@@ -3452,26 +3452,26 @@
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Service Degradation</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>2026-04-07T18:03:00Z</t>
+          <t>2026-04-09T18:04:00Z</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Apr 07, 2026 7:21 PM GMT</t>
+          <t>Apr 09, 2026 9:35 PM GMT</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>78</v>
+        <v>211</v>
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
@@ -3482,26 +3482,26 @@
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-08T04:10:00Z</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
@@ -3512,26 +3512,26 @@
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>2026-04-02T00:27:00Z</t>
+          <t>2026-04-08T04:09:00Z</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Apr 02, 2026 1:17 AM GMT</t>
+          <t>Apr 08, 2026 4:12 AM GMT</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E84" s="5" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
@@ -3542,17 +3542,17 @@
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Service Degradation</t>
         </is>
       </c>
       <c r="B85" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-07T18:03:00Z</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 07, 2026 7:21 PM GMT</t>
         </is>
       </c>
       <c r="D85" s="5" t="inlineStr">
@@ -3561,11 +3561,11 @@
         </is>
       </c>
       <c r="E85" s="5" t="n">
-        <v>203</v>
+        <v>78</v>
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -3577,25 +3577,25 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>2026-03-26T03:52:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 7:15 AM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E86" s="5" t="n">
-        <v>203</v>
+        <v>50</v>
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -3607,25 +3607,25 @@
       </c>
       <c r="B87" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-04-02T00:27:00Z</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Apr 02, 2026 1:17 AM GMT</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E87" s="5" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-04</t>
         </is>
       </c>
     </row>
@@ -3637,21 +3637,21 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T23:07:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Mar 26, 2026 1:37 AM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E88" s="5" t="n">
-        <v>150</v>
+        <v>203</v>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
@@ -3667,21 +3667,21 @@
       </c>
       <c r="B89" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-26T03:52:00Z</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 7:15 AM GMT</t>
         </is>
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E89" s="5" t="n">
-        <v>123</v>
+        <v>203</v>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
@@ -3697,21 +3697,21 @@
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E90" s="5" t="n">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
@@ -3727,21 +3727,21 @@
       </c>
       <c r="B91" s="5" t="inlineStr">
         <is>
-          <t>2026-03-25T14:07:00Z</t>
+          <t>2026-03-25T23:07:00Z</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Mar 25, 2026 4:10 PM GMT</t>
+          <t>Mar 26, 2026 1:37 AM GMT</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E91" s="5" t="n">
-        <v>123</v>
+        <v>150</v>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
@@ -3767,7 +3767,7 @@
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E92" s="5" t="n">
@@ -3787,21 +3787,21 @@
       </c>
       <c r="B93" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T21:04:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 10:34 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D93" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
@@ -3817,21 +3817,21 @@
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>2026-03-20T17:44:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Mar 20, 2026 6:26 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E94" s="5" t="n">
-        <v>42</v>
+        <v>123</v>
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
@@ -3847,21 +3847,21 @@
       </c>
       <c r="B95" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-03-25T14:07:00Z</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Mar 25, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E95" s="5" t="n">
-        <v>99</v>
+        <v>123</v>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
@@ -3877,21 +3877,21 @@
       </c>
       <c r="B96" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T19:11:00Z</t>
+          <t>2026-03-20T21:04:00Z</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 8:50 PM GMT</t>
+          <t>Mar 20, 2026 10:34 PM GMT</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E96" s="5" t="n">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
@@ -3902,26 +3902,26 @@
     <row r="97">
       <c r="A97" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B97" s="5" t="inlineStr">
         <is>
-          <t>2026-03-18T00:43:00Z</t>
+          <t>2026-03-20T17:44:00Z</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 12:46 AM GMT</t>
+          <t>Mar 20, 2026 6:26 PM GMT</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E97" s="5" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
@@ -3937,21 +3937,21 @@
       </c>
       <c r="B98" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E98" s="5" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
@@ -3967,21 +3967,21 @@
       </c>
       <c r="B99" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T22:16:00Z</t>
+          <t>2026-03-18T19:11:00Z</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
         <is>
-          <t>Mar 18, 2026 1:34 AM GMT</t>
+          <t>Mar 18, 2026 8:50 PM GMT</t>
         </is>
       </c>
       <c r="D99" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E99" s="5" t="n">
-        <v>198</v>
+        <v>99</v>
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
@@ -3997,21 +3997,21 @@
       </c>
       <c r="B100" s="5" t="inlineStr">
         <is>
-          <t>2026-03-17T19:46:00Z</t>
+          <t>2026-03-18T00:43:00Z</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
         <is>
-          <t>Mar 17, 2026 7:48 PM GMT</t>
+          <t>Mar 18, 2026 12:46 AM GMT</t>
         </is>
       </c>
       <c r="D100" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E100" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
@@ -4022,26 +4022,26 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B101" s="5" t="inlineStr">
         <is>
-          <t>2026-03-13T00:37:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
         <is>
-          <t>Mar 13, 2026 12:41 AM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D101" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E101" s="5" t="n">
-        <v>4</v>
+        <v>198</v>
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
@@ -4052,26 +4052,26 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B102" s="5" t="inlineStr">
         <is>
-          <t>2026-03-11T23:50:00Z</t>
+          <t>2026-03-17T22:16:00Z</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
         <is>
-          <t>Mar 11, 2026 11:54 PM GMT</t>
+          <t>Mar 18, 2026 1:34 AM GMT</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E102" s="5" t="n">
-        <v>4</v>
+        <v>198</v>
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
@@ -4082,26 +4082,26 @@
     <row r="103">
       <c r="A103" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B103" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-17T19:46:00Z</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 17, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E103" s="5" t="n">
-        <v>164</v>
+        <v>2</v>
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
@@ -4112,26 +4112,26 @@
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B104" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T05:01:00Z</t>
+          <t>2026-03-13T00:37:00Z</t>
         </is>
       </c>
       <c r="C104" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 7:45 AM GMT</t>
+          <t>Mar 13, 2026 12:41 AM GMT</t>
         </is>
       </c>
       <c r="D104" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E104" s="5" t="n">
-        <v>164</v>
+        <v>4</v>
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
@@ -4142,26 +4142,26 @@
     <row r="105">
       <c r="A105" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B105" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-11T23:50:00Z</t>
         </is>
       </c>
       <c r="C105" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 11, 2026 11:54 PM GMT</t>
         </is>
       </c>
       <c r="D105" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E105" s="5" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
@@ -4177,21 +4177,21 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>2026-03-05T01:20:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C106" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 2:45 AM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D106" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E106" s="5" t="n">
-        <v>85</v>
+        <v>164</v>
       </c>
       <c r="F106" s="5" t="inlineStr">
         <is>
@@ -4207,21 +4207,21 @@
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-05T05:01:00Z</t>
         </is>
       </c>
       <c r="C107" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 05, 2026 7:45 AM GMT</t>
         </is>
       </c>
       <c r="D107" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E107" s="5" t="n">
-        <v>87</v>
+        <v>164</v>
       </c>
       <c r="F107" s="5" t="inlineStr">
         <is>
@@ -4237,21 +4237,21 @@
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T23:49:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C108" s="5" t="inlineStr">
         <is>
-          <t>Mar 05, 2026 1:16 AM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D108" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E108" s="5" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
@@ -4267,21 +4267,21 @@
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-05T01:20:00Z</t>
         </is>
       </c>
       <c r="C109" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 2:45 AM GMT</t>
         </is>
       </c>
       <c r="D109" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E109" s="5" t="n">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
@@ -4297,21 +4297,21 @@
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C110" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D110" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E110" s="5" t="n">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
@@ -4327,21 +4327,21 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>2026-03-04T14:35:00Z</t>
+          <t>2026-03-04T23:49:00Z</t>
         </is>
       </c>
       <c r="C111" s="5" t="inlineStr">
         <is>
-          <t>Mar 04, 2026 4:10 PM GMT</t>
+          <t>Mar 05, 2026 1:16 AM GMT</t>
         </is>
       </c>
       <c r="D111" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E111" s="5" t="n">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
@@ -4367,7 +4367,7 @@
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E112" s="5" t="n">
@@ -4382,26 +4382,26 @@
     <row r="113">
       <c r="A113" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B113" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C113" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 5:02 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E113" s="5" t="n">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
@@ -4412,26 +4412,26 @@
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B114" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T16:51:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C114" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 4:56 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E114" s="5" t="n">
-        <v>5</v>
+        <v>95</v>
       </c>
       <c r="F114" s="5" t="inlineStr">
         <is>
@@ -4442,26 +4442,26 @@
     <row r="115">
       <c r="A115" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B115" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:44:00Z</t>
+          <t>2026-03-04T14:35:00Z</t>
         </is>
       </c>
       <c r="C115" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 3:15 PM GMT</t>
+          <t>Mar 04, 2026 4:10 PM GMT</t>
         </is>
       </c>
       <c r="D115" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E115" s="5" t="n">
-        <v>31</v>
+        <v>95</v>
       </c>
       <c r="F115" s="5" t="inlineStr">
         <is>
@@ -4477,21 +4477,21 @@
       </c>
       <c r="B116" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:42:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C116" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:44 PM GMT</t>
+          <t>Mar 02, 2026 5:02 PM GMT</t>
         </is>
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E116" s="5" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="F116" s="5" t="inlineStr">
         <is>
@@ -4507,21 +4507,21 @@
       </c>
       <c r="B117" s="5" t="inlineStr">
         <is>
-          <t>2026-03-02T14:41:00Z</t>
+          <t>2026-03-02T16:51:00Z</t>
         </is>
       </c>
       <c r="C117" s="5" t="inlineStr">
         <is>
-          <t>Mar 02, 2026 2:42 PM GMT</t>
+          <t>Mar 02, 2026 4:56 PM GMT</t>
         </is>
       </c>
       <c r="D117" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E117" s="5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F117" s="5" t="inlineStr">
         <is>
@@ -4537,111 +4537,111 @@
       </c>
       <c r="B118" s="5" t="inlineStr">
         <is>
-          <t>2026-02-26T16:39:00Z</t>
+          <t>2026-03-02T14:44:00Z</t>
         </is>
       </c>
       <c r="C118" s="5" t="inlineStr">
         <is>
-          <t>Feb 26, 2026 4:44 PM GMT</t>
+          <t>Mar 02, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E118" s="5" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="F118" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B119" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-02T14:42:00Z</t>
         </is>
       </c>
       <c r="C119" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 02, 2026 2:44 PM GMT</t>
         </is>
       </c>
       <c r="D119" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - APAC</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E119" s="5" t="n">
-        <v>207</v>
+        <v>2</v>
       </c>
       <c r="F119" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>2026-02-20T15:28:00Z</t>
+          <t>2026-03-02T14:41:00Z</t>
         </is>
       </c>
       <c r="C120" s="5" t="inlineStr">
         <is>
-          <t>Feb 20, 2026 6:55 PM GMT</t>
+          <t>Mar 02, 2026 2:42 PM GMT</t>
         </is>
       </c>
       <c r="D120" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - APAC</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E120" s="5" t="n">
-        <v>207</v>
+        <v>1</v>
       </c>
       <c r="F120" s="5" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-03</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B121" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-02-26T16:39:00Z</t>
         </is>
       </c>
       <c r="C121" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Feb 26, 2026 4:44 PM GMT</t>
         </is>
       </c>
       <c r="D121" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E121" s="5" t="n">
-        <v>159</v>
+        <v>5</v>
       </c>
       <c r="F121" s="5" t="inlineStr">
         <is>
@@ -4657,21 +4657,21 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>2026-02-18T19:36:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C122" s="5" t="inlineStr">
         <is>
-          <t>Feb 18, 2026 10:15 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D122" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - APAC</t>
         </is>
       </c>
       <c r="E122" s="5" t="n">
-        <v>159</v>
+        <v>207</v>
       </c>
       <c r="F122" s="5" t="inlineStr">
         <is>
@@ -4682,26 +4682,26 @@
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B123" s="5" t="inlineStr">
         <is>
-          <t>2026-02-15T19:46:00Z</t>
+          <t>2026-02-20T15:28:00Z</t>
         </is>
       </c>
       <c r="C123" s="5" t="inlineStr">
         <is>
-          <t>Feb 15, 2026 7:48 PM GMT</t>
+          <t>Feb 20, 2026 6:55 PM GMT</t>
         </is>
       </c>
       <c r="D123" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand API - APAC</t>
         </is>
       </c>
       <c r="E123" s="5" t="n">
-        <v>2</v>
+        <v>207</v>
       </c>
       <c r="F123" s="5" t="inlineStr">
         <is>
@@ -4712,26 +4712,26 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B124" s="5" t="inlineStr">
         <is>
-          <t>2026-02-14T22:07:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C124" s="5" t="inlineStr">
         <is>
-          <t>Feb 14, 2026 10:09 PM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D124" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E124" s="5" t="n">
-        <v>2</v>
+        <v>159</v>
       </c>
       <c r="F124" s="5" t="inlineStr">
         <is>
@@ -4747,21 +4747,21 @@
       </c>
       <c r="B125" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-02-18T19:36:00Z</t>
         </is>
       </c>
       <c r="C125" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Feb 18, 2026 10:15 PM GMT</t>
         </is>
       </c>
       <c r="D125" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - SGP</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E125" s="5" t="n">
-        <v>282</v>
+        <v>159</v>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
@@ -4772,26 +4772,26 @@
     <row r="126">
       <c r="A126" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B126" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T16:28:00Z</t>
+          <t>2026-02-15T19:46:00Z</t>
         </is>
       </c>
       <c r="C126" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 9:10 PM GMT</t>
+          <t>Feb 15, 2026 7:48 PM GMT</t>
         </is>
       </c>
       <c r="D126" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - SGP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E126" s="5" t="n">
-        <v>282</v>
+        <v>2</v>
       </c>
       <c r="F126" s="5" t="inlineStr">
         <is>
@@ -4802,26 +4802,26 @@
     <row r="127">
       <c r="A127" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B127" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-02-14T22:07:00Z</t>
         </is>
       </c>
       <c r="C127" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Feb 14, 2026 10:09 PM GMT</t>
         </is>
       </c>
       <c r="D127" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E127" s="5" t="n">
-        <v>127</v>
+        <v>2</v>
       </c>
       <c r="F127" s="5" t="inlineStr">
         <is>
@@ -4837,21 +4837,21 @@
       </c>
       <c r="B128" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T04:56:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C128" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 7:03 AM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D128" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand Tenant Portal - SGP</t>
         </is>
       </c>
       <c r="E128" s="5" t="n">
-        <v>127</v>
+        <v>282</v>
       </c>
       <c r="F128" s="5" t="inlineStr">
         <is>
@@ -4867,21 +4867,21 @@
       </c>
       <c r="B129" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-02-05T16:28:00Z</t>
         </is>
       </c>
       <c r="C129" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Feb 05, 2026 9:10 PM GMT</t>
         </is>
       </c>
       <c r="D129" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand API - SGP</t>
         </is>
       </c>
       <c r="E129" s="5" t="n">
-        <v>98</v>
+        <v>282</v>
       </c>
       <c r="F129" s="5" t="inlineStr">
         <is>
@@ -4897,21 +4897,21 @@
       </c>
       <c r="B130" s="5" t="inlineStr">
         <is>
-          <t>2026-02-05T01:57:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C130" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 3:35 AM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D130" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E130" s="5" t="n">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="F130" s="5" t="inlineStr">
         <is>
@@ -4927,21 +4927,21 @@
       </c>
       <c r="B131" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-05T04:56:00Z</t>
         </is>
       </c>
       <c r="C131" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 05, 2026 7:03 AM GMT</t>
         </is>
       </c>
       <c r="D131" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E131" s="5" t="n">
-        <v>88</v>
+        <v>127</v>
       </c>
       <c r="F131" s="5" t="inlineStr">
         <is>
@@ -4957,21 +4957,21 @@
       </c>
       <c r="B132" s="5" t="inlineStr">
         <is>
-          <t>2026-02-04T23:58:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C132" s="5" t="inlineStr">
         <is>
-          <t>Feb 05, 2026 1:26 AM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D132" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E132" s="5" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F132" s="5" t="inlineStr">
         <is>
@@ -4987,25 +4987,25 @@
       </c>
       <c r="B133" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-05T01:57:00Z</t>
         </is>
       </c>
       <c r="C133" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 05, 2026 3:35 AM GMT</t>
         </is>
       </c>
       <c r="D133" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E133" s="5" t="n">
-        <v>4234</v>
+        <v>98</v>
       </c>
       <c r="F133" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
@@ -5017,81 +5017,81 @@
       </c>
       <c r="B134" s="5" t="inlineStr">
         <is>
-          <t>2026-01-30T19:08:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C134" s="5" t="inlineStr">
         <is>
-          <t>Feb 02, 2026 5:42 PM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D134" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - EMEA</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E134" s="5" t="n">
-        <v>4234</v>
+        <v>88</v>
       </c>
       <c r="F134" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B135" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:46:00Z</t>
+          <t>2026-02-04T23:58:00Z</t>
         </is>
       </c>
       <c r="C135" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:47 PM GMT</t>
+          <t>Feb 05, 2026 1:26 AM GMT</t>
         </is>
       </c>
       <c r="D135" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E135" s="5" t="n">
-        <v>1</v>
+        <v>88</v>
       </c>
       <c r="F135" s="5" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-02</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B136" s="5" t="inlineStr">
         <is>
-          <t>2026-01-27T14:45:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C136" s="5" t="inlineStr">
         <is>
-          <t>Jan 27, 2026 2:46 PM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D136" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
         </is>
       </c>
       <c r="E136" s="5" t="n">
-        <v>1</v>
+        <v>4234</v>
       </c>
       <c r="F136" s="5" t="inlineStr">
         <is>
@@ -5107,21 +5107,21 @@
       </c>
       <c r="B137" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-01-30T19:08:00Z</t>
         </is>
       </c>
       <c r="C137" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Feb 02, 2026 5:42 PM GMT</t>
         </is>
       </c>
       <c r="D137" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
       <c r="E137" s="5" t="n">
-        <v>1595</v>
+        <v>4234</v>
       </c>
       <c r="F137" s="5" t="inlineStr">
         <is>
@@ -5132,26 +5132,26 @@
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B138" s="5" t="inlineStr">
         <is>
-          <t>2026-01-23T23:57:00Z</t>
+          <t>2026-01-27T14:46:00Z</t>
         </is>
       </c>
       <c r="C138" s="5" t="inlineStr">
         <is>
-          <t>Jan 25, 2026 2:32 AM GMT</t>
+          <t>Jan 27, 2026 2:47 PM GMT</t>
         </is>
       </c>
       <c r="D138" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand API - FedRAMP</t>
         </is>
       </c>
       <c r="E138" s="5" t="n">
-        <v>1595</v>
+        <v>1</v>
       </c>
       <c r="F138" s="5" t="inlineStr">
         <is>
@@ -5162,26 +5162,26 @@
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B139" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T16:24:00Z</t>
+          <t>2026-01-27T14:45:00Z</t>
         </is>
       </c>
       <c r="C139" s="5" t="inlineStr">
         <is>
-          <t>Jan 20, 2026 3:26 AM GMT</t>
+          <t>Jan 27, 2026 2:46 PM GMT</t>
         </is>
       </c>
       <c r="D139" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
         </is>
       </c>
       <c r="E139" s="5" t="n">
-        <v>4982</v>
+        <v>1</v>
       </c>
       <c r="F139" s="5" t="inlineStr">
         <is>
@@ -5192,26 +5192,26 @@
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B140" s="5" t="inlineStr">
         <is>
-          <t>2026-01-16T15:14:00Z</t>
+          <t>2026-01-23T23:57:00Z</t>
         </is>
       </c>
       <c r="C140" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:15 PM GMT</t>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
         </is>
       </c>
       <c r="D140" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / eu-sast-aviator</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E140" s="5" t="n">
-        <v>1</v>
+        <v>1595</v>
       </c>
       <c r="F140" s="5" t="inlineStr">
         <is>
@@ -5227,21 +5227,21 @@
       </c>
       <c r="B141" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T21:13:00Z</t>
+          <t>2026-01-23T23:57:00Z</t>
         </is>
       </c>
       <c r="C141" s="5" t="inlineStr">
         <is>
-          <t>Jan 16, 2026 3:03 PM GMT</t>
+          <t>Jan 25, 2026 2:32 AM GMT</t>
         </is>
       </c>
       <c r="D141" s="5" t="inlineStr">
         <is>
-          <t>SAST Aviator / ams-sast-aviator</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E141" s="5" t="n">
-        <v>1070</v>
+        <v>1595</v>
       </c>
       <c r="F141" s="5" t="inlineStr">
         <is>
@@ -5252,26 +5252,26 @@
     <row r="142">
       <c r="A142" s="5" t="inlineStr">
         <is>
-          <t>Outage</t>
+          <t>Maintenance</t>
         </is>
       </c>
       <c r="B142" s="5" t="inlineStr">
         <is>
-          <t>2026-01-15T04:24:00Z</t>
+          <t>2026-01-16T16:24:00Z</t>
         </is>
       </c>
       <c r="C142" s="5" t="inlineStr">
         <is>
-          <t>Jan 15, 2026 4:25 AM GMT</t>
+          <t>Jan 20, 2026 3:26 AM GMT</t>
         </is>
       </c>
       <c r="D142" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand - Vulncat</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E142" s="5" t="n">
-        <v>1</v>
+        <v>4982</v>
       </c>
       <c r="F142" s="5" t="inlineStr">
         <is>
@@ -5287,12 +5287,12 @@
       </c>
       <c r="B143" s="5" t="inlineStr">
         <is>
-          <t>2026-01-10T15:08:00Z</t>
+          <t>2026-01-16T15:14:00Z</t>
         </is>
       </c>
       <c r="C143" s="5" t="inlineStr">
         <is>
-          <t>Jan 10, 2026 3:10 PM GMT</t>
+          <t>Jan 16, 2026 3:15 PM GMT</t>
         </is>
       </c>
       <c r="D143" s="5" t="inlineStr">
@@ -5301,7 +5301,7 @@
         </is>
       </c>
       <c r="E143" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F143" s="5" t="inlineStr">
         <is>
@@ -5317,21 +5317,21 @@
       </c>
       <c r="B144" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-01-15T21:13:00Z</t>
         </is>
       </c>
       <c r="C144" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Jan 16, 2026 3:03 PM GMT</t>
         </is>
       </c>
       <c r="D144" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - AMS</t>
+          <t>SAST Aviator / ams-sast-aviator</t>
         </is>
       </c>
       <c r="E144" s="5" t="n">
-        <v>140</v>
+        <v>1070</v>
       </c>
       <c r="F144" s="5" t="inlineStr">
         <is>
@@ -5342,26 +5342,26 @@
     <row r="145">
       <c r="A145" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B145" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T04:54:00Z</t>
+          <t>2026-01-15T04:24:00Z</t>
         </is>
       </c>
       <c r="C145" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 7:14 AM GMT</t>
+          <t>Jan 15, 2026 4:25 AM GMT</t>
         </is>
       </c>
       <c r="D145" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - AMS</t>
+          <t>Fortify on Demand - Vulncat</t>
         </is>
       </c>
       <c r="E145" s="5" t="n">
-        <v>140</v>
+        <v>1</v>
       </c>
       <c r="F145" s="5" t="inlineStr">
         <is>
@@ -5372,26 +5372,26 @@
     <row r="146">
       <c r="A146" s="5" t="inlineStr">
         <is>
-          <t>Maintenance</t>
+          <t>Outage</t>
         </is>
       </c>
       <c r="B146" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-10T15:08:00Z</t>
         </is>
       </c>
       <c r="C146" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Jan 10, 2026 3:10 PM GMT</t>
         </is>
       </c>
       <c r="D146" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+          <t>SAST Aviator / eu-sast-aviator</t>
         </is>
       </c>
       <c r="E146" s="5" t="n">
-        <v>137</v>
+        <v>2</v>
       </c>
       <c r="F146" s="5" t="inlineStr">
         <is>
@@ -5407,21 +5407,21 @@
       </c>
       <c r="B147" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T01:13:00Z</t>
+          <t>2026-01-08T04:54:00Z</t>
         </is>
       </c>
       <c r="C147" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 3:30 AM GMT</t>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
         </is>
       </c>
       <c r="D147" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand API - FedRAMP</t>
+          <t>Fortify on Demand Tenant Portal - AMS</t>
         </is>
       </c>
       <c r="E147" s="5" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F147" s="5" t="inlineStr">
         <is>
@@ -5437,21 +5437,21 @@
       </c>
       <c r="B148" s="5" t="inlineStr">
         <is>
-          <t>2026-01-08T00:24:00Z</t>
+          <t>2026-01-08T04:54:00Z</t>
         </is>
       </c>
       <c r="C148" s="5" t="inlineStr">
         <is>
-          <t>Jan 08, 2026 1:02 AM GMT</t>
+          <t>Jan 08, 2026 7:14 AM GMT</t>
         </is>
       </c>
       <c r="D148" s="5" t="inlineStr">
         <is>
-          <t>Fortify on Demand Tenant Portal - EMEA</t>
+          <t>Fortify on Demand API - AMS</t>
         </is>
       </c>
       <c r="E148" s="5" t="n">
-        <v>38</v>
+        <v>140</v>
       </c>
       <c r="F148" s="5" t="inlineStr">
         <is>
@@ -5467,32 +5467,122 @@
       </c>
       <c r="B149" s="5" t="inlineStr">
         <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T01:13:00Z</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 3:30 AM GMT</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand API - FedRAMP</t>
+        </is>
+      </c>
+      <c r="E150" s="5" t="n">
+        <v>137</v>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
           <t>2026-01-08T00:24:00Z</t>
         </is>
       </c>
-      <c r="C149" s="5" t="inlineStr">
+      <c r="C151" s="5" t="inlineStr">
         <is>
           <t>Jan 08, 2026 1:02 AM GMT</t>
         </is>
       </c>
-      <c r="D149" s="5" t="inlineStr">
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>Fortify on Demand Tenant Portal - EMEA</t>
+        </is>
+      </c>
+      <c r="E151" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-08T00:24:00Z</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>Jan 08, 2026 1:02 AM GMT</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
         <is>
           <t>Fortify on Demand API - EMEA</t>
         </is>
       </c>
-      <c r="E149" s="5" t="n">
+      <c r="E152" s="5" t="n">
         <v>38</v>
       </c>
-      <c r="F149" s="5" t="inlineStr">
+      <c r="F152" s="5" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="11" t="inlineStr">
-        <is>
-          <t>Report revised: July 02, 2026</t>
+    <row r="153">
+      <c r="A153" s="11" t="inlineStr">
+        <is>
+          <t>Report revised: July 16, 2026</t>
         </is>
       </c>
     </row>
@@ -5945,7 +6035,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Last updated: July 2, 2026 (Jun 2026 finalized: 2 outages (EU SAST Aviator Jun 8 2 min, AMS SAST Aviator Jun 9 2 min), 4 total outage minutes, 99.9907% uptime; new maintenance events Jun 4-5, 22-27 added; AMS service degradation Jun 11-Jun 25 recorded; times converted from BST to GMT).</t>
+          <t>Last updated: July 16, 2026 (mid-month snapshot for Jul 2026 through Jul 16; 3 outages added: Jul 6 APAC Portal 6 min, Jul 7 APAC API 7 min, Jul 8 AMS SAST Aviator 4 min; all times converted from BST to GMT; Jun 2026 previously finalized July 2, 2026).</t>
         </is>
       </c>
     </row>
@@ -6632,7 +6722,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>Last updated: July 2, 2026</t>
+          <t>Last updated: July 16, 2026</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7231,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>1</v>
+        <v>0.9998655913978495</v>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
@@ -7197,7 +7287,7 @@
         <v>1</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>1</v>
+        <v>0.9998431899641577</v>
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
@@ -7556,7 +7646,7 @@
         <v>0.9999537037037037</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>1</v>
+        <v>0.999910394265233</v>
       </c>
       <c r="I20" s="14" t="inlineStr">
         <is>
@@ -9835,7 +9925,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Month in progress. Will be finalized after July 31, 2026.</t>
+          <t>Month in progress (partial through July 16, 2026). Will be finalized after July 31, 2026.</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9968,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -9890,7 +9980,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>17</t>
         </is>
       </c>
     </row>

</xml_diff>